<commit_message>
prob1234 finish | prob5 50%
</commit_message>
<xml_diff>
--- a/4/FY3/FY3_optimization_results/best_solution.xlsx
+++ b/4/FY3/FY3_optimization_results/best_solution.xlsx
@@ -487,37 +487,37 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>74.5</v>
+        <v>76.5</v>
       </c>
       <c r="B2" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>6820.956291312405</v>
+        <v>6708.740124666529</v>
       </c>
       <c r="F2" t="n">
-        <v>-39.72724774311018</v>
+        <v>-47.88492167265395</v>
       </c>
       <c r="G2" t="n">
         <v>700</v>
       </c>
       <c r="H2" t="n">
-        <v>6855.162803450422</v>
+        <v>6739.554912695508</v>
       </c>
       <c r="I2" t="n">
-        <v>83.61745026759355</v>
+        <v>80.46790781983935</v>
       </c>
       <c r="J2" t="n">
         <v>695.1</v>
       </c>
       <c r="K2" t="n">
-        <v>3.099999999999998</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>